<commit_message>
fix(dashboard): Sincronização dinâmica de todas as 66 praças nos filtros e backoff rigoroso para 429 no SharePoint
</commit_message>
<xml_diff>
--- a/Controle_Frota_Capture_Sites_400.xlsx
+++ b/Controle_Frota_Capture_Sites_400.xlsx
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>3</v>
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>3</v>
@@ -709,15 +709,19 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="3" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Rede Globo, Record TV, SBT BKP</t>
+        </is>
+      </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -768,15 +772,19 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="5" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Rede Globo, Record TV, SBT BKP</t>
+        </is>
+      </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -827,7 +835,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>0</v>
@@ -886,7 +894,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>0</v>
@@ -1193,7 +1201,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>2</v>
@@ -1256,7 +1264,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>0</v>
@@ -1318,11 +1326,11 @@
         <v>13</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Rede Globo, Rede Globo</t>
+          <t>Rede Globo</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
@@ -1378,7 +1386,7 @@
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H15" s="4" t="n">
         <v>0</v>
@@ -1437,7 +1445,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>0</v>
@@ -1622,7 +1630,7 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H19" s="4" t="n">
         <v>0</v>
@@ -1681,7 +1689,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>0</v>
@@ -1740,7 +1748,7 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>0</v>
@@ -1799,7 +1807,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>4</v>
@@ -1862,7 +1870,7 @@
         </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H23" s="4" t="n">
         <v>0</v>
@@ -1921,7 +1929,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>0</v>
@@ -2039,7 +2047,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>0</v>
@@ -2157,7 +2165,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>0</v>
@@ -2216,15 +2224,19 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="5" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Rede TV, Rede Globo, Record TV, Rede Bandeirantes (+4)</t>
+        </is>
+      </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -2275,7 +2287,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>0</v>
@@ -2334,7 +2346,7 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H31" s="4" t="n">
         <v>0</v>
@@ -2393,7 +2405,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>0</v>
@@ -2452,7 +2464,7 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H33" s="4" t="n">
         <v>4</v>
@@ -2515,7 +2527,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>0</v>
@@ -2574,7 +2586,7 @@
         </is>
       </c>
       <c r="G35" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H35" s="4" t="n">
         <v>0</v>
@@ -2619,7 +2631,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>CS 1</t>
+          <t>CS 2</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2633,7 +2645,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>0</v>
@@ -2692,7 +2704,7 @@
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H37" s="4" t="n">
         <v>0</v>
@@ -2810,7 +2822,7 @@
         </is>
       </c>
       <c r="G39" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H39" s="4" t="n">
         <v>1</v>
@@ -2873,7 +2885,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H40" s="2" t="n">
         <v>0</v>
@@ -2932,7 +2944,7 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H41" s="4" t="n">
         <v>0</v>
@@ -2991,7 +3003,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H42" s="2" t="n">
         <v>0</v>
@@ -3050,7 +3062,7 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H43" s="4" t="n">
         <v>0</v>
@@ -3109,7 +3121,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H44" s="2" t="n">
         <v>0</v>
@@ -3168,7 +3180,7 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H45" s="4" t="n">
         <v>0</v>
@@ -3227,7 +3239,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>0</v>
@@ -3286,7 +3298,7 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H47" s="4" t="n">
         <v>0</v>
@@ -3345,7 +3357,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H48" s="2" t="n">
         <v>0</v>
@@ -3404,7 +3416,7 @@
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H49" s="4" t="n">
         <v>0</v>
@@ -3522,7 +3534,7 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H51" s="4" t="n">
         <v>0</v>
@@ -3581,7 +3593,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H52" s="2" t="n">
         <v>0</v>
@@ -3825,7 +3837,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H56" s="2" t="n">
         <v>0</v>
@@ -3884,7 +3896,7 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H57" s="4" t="n">
         <v>0</v>
@@ -3943,7 +3955,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H58" s="2" t="n">
         <v>2</v>
@@ -4006,7 +4018,7 @@
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H59" s="4" t="n">
         <v>0</v>
@@ -4065,7 +4077,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H60" s="2" t="n">
         <v>0</v>
@@ -4127,12 +4139,16 @@
         <v>18</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>Rede Globo</t>
+        </is>
+      </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
@@ -4183,7 +4199,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H62" s="2" t="n">
         <v>0</v>
@@ -4242,7 +4258,7 @@
         </is>
       </c>
       <c r="G63" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H63" s="4" t="n">
         <v>0</v>
@@ -4304,12 +4320,16 @@
         <v>15</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I64" s="3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Rede Globo</t>
+        </is>
+      </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
@@ -4360,15 +4380,19 @@
         </is>
       </c>
       <c r="G65" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" s="5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>Rede Globo, Rede TV</t>
+        </is>
+      </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
@@ -4419,7 +4443,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H66" s="2" t="n">
         <v>0</v>
@@ -4604,7 +4628,7 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="H69" s="4" t="n">
         <v>0</v>
@@ -4663,15 +4687,19 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" s="3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>Rede Globo, SBT</t>
+        </is>
+      </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
@@ -4722,7 +4750,7 @@
         </is>
       </c>
       <c r="G71" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H71" s="4" t="n">
         <v>0</v>
@@ -4781,7 +4809,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H72" s="2" t="n">
         <v>0</v>
@@ -4840,7 +4868,7 @@
         </is>
       </c>
       <c r="G73" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H73" s="4" t="n">
         <v>0</v>
@@ -4899,7 +4927,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H74" s="2" t="n">
         <v>0</v>
@@ -4944,7 +4972,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>CS 2</t>
+          <t>CS 1</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -4958,7 +4986,7 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H75" s="4" t="n">
         <v>0</v>
@@ -5017,7 +5045,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H76" s="2" t="n">
         <v>0</v>
@@ -5076,7 +5104,7 @@
         </is>
       </c>
       <c r="G77" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H77" s="4" t="n">
         <v>0</v>
@@ -5135,7 +5163,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H78" s="2" t="n">
         <v>9</v>
@@ -5257,7 +5285,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H80" s="2" t="n">
         <v>0</v>
@@ -5316,15 +5344,19 @@
         </is>
       </c>
       <c r="G81" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H81" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>Rede Globo</t>
+        </is>
+      </c>
       <c r="J81" s="5" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K81" s="5" t="inlineStr">
@@ -5434,7 +5466,7 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H83" s="4" t="n">
         <v>0</v>
@@ -5493,7 +5525,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H84" s="2" t="n">
         <v>0</v>
@@ -5611,7 +5643,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H86" s="2" t="n">
         <v>0</v>
@@ -5670,7 +5702,7 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H87" s="4" t="n">
         <v>0</v>
@@ -5729,7 +5761,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H88" s="2" t="n">
         <v>0</v>
@@ -5788,7 +5820,7 @@
         </is>
       </c>
       <c r="G89" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H89" s="4" t="n">
         <v>0</v>
@@ -5906,7 +5938,7 @@
         </is>
       </c>
       <c r="G91" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H91" s="4" t="n">
         <v>22</v>
@@ -5969,7 +6001,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H92" s="2" t="n">
         <v>0</v>
@@ -6028,7 +6060,7 @@
         </is>
       </c>
       <c r="G93" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H93" s="4" t="n">
         <v>0</v>
@@ -6150,7 +6182,7 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H95" s="4" t="n">
         <v>4</v>
@@ -6213,15 +6245,19 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I96" s="3" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>Rede Globo, Record TV, SBT BKP</t>
+        </is>
+      </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
@@ -6338,12 +6374,16 @@
         <v>14</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I98" s="3" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>Rede Globo, Record TV, Rede Bandeirantes, TV Brasil (+3)</t>
+        </is>
+      </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K98" s="3" t="inlineStr">
@@ -6394,7 +6434,7 @@
         </is>
       </c>
       <c r="G99" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H99" s="4" t="n">
         <v>0</v>
@@ -6512,15 +6552,19 @@
         </is>
       </c>
       <c r="G101" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H101" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I101" s="5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>Rede Globo, Rede TV</t>
+        </is>
+      </c>
       <c r="J101" s="5" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K101" s="5" t="inlineStr">
@@ -6630,7 +6674,7 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H103" s="4" t="n">
         <v>0</v>
@@ -6689,7 +6733,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H104" s="2" t="n">
         <v>0</v>
@@ -6748,7 +6792,7 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H105" s="4" t="n">
         <v>0</v>
@@ -6793,7 +6837,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>CS 2</t>
+          <t>CS 1</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -6807,15 +6851,19 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I106" s="3" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>Rede Globo, Record TV, Saudade FM, Hot 98 fm (+4)</t>
+        </is>
+      </c>
       <c r="J106" s="3" t="inlineStr">
         <is>
-          <t>TBS DTV / MCR</t>
+          <t>TBS DTV (ISDB-Tb UHF)</t>
         </is>
       </c>
       <c r="K106" s="3" t="inlineStr">
@@ -6866,7 +6914,7 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H107" s="4" t="n">
         <v>0</v>
@@ -6925,7 +6973,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H108" s="2" t="n">
         <v>0</v>
@@ -6984,7 +7032,7 @@
         </is>
       </c>
       <c r="G109" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H109" s="4" t="n">
         <v>2</v>
@@ -7047,7 +7095,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H110" s="2" t="n">
         <v>2</v>
@@ -7110,7 +7158,7 @@
         </is>
       </c>
       <c r="G111" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H111" s="4" t="n">
         <v>0</v>
@@ -7169,7 +7217,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H112" s="2" t="n">
         <v>2</v>
@@ -7232,7 +7280,7 @@
         </is>
       </c>
       <c r="G113" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H113" s="4" t="n">
         <v>0</v>
@@ -7291,7 +7339,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H114" s="2" t="n">
         <v>0</v>
@@ -7476,7 +7524,7 @@
         </is>
       </c>
       <c r="G117" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H117" s="4" t="n">
         <v>0</v>
@@ -7535,7 +7583,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H118" s="2" t="n">
         <v>0</v>
@@ -7580,7 +7628,7 @@
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>CS 1</t>
+          <t>CS 2</t>
         </is>
       </c>
       <c r="E119" s="4" t="inlineStr">
@@ -7594,19 +7642,15 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H119" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I119" s="5" t="inlineStr">
-        <is>
-          <t>Rede Bandeirantes BKP, Rede Globo BKP, Rede Globo, Rede Bandeirantes</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I119" s="5" t="inlineStr"/>
       <c r="J119" s="5" t="inlineStr">
         <is>
-          <t>Streaming IP / FM + TBS DTV (ISDB-Tb UHF)</t>
+          <t>TBS DTV / MCR</t>
         </is>
       </c>
       <c r="K119" s="5" t="inlineStr">
@@ -7657,7 +7701,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H120" s="2" t="n">
         <v>0</v>
@@ -7716,7 +7760,7 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H121" s="4" t="n">
         <v>0</v>
@@ -7775,7 +7819,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H122" s="2" t="n">
         <v>2</v>
@@ -7838,7 +7882,7 @@
         </is>
       </c>
       <c r="G123" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H123" s="4" t="n">
         <v>2</v>
@@ -7901,7 +7945,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H124" s="2" t="n">
         <v>2</v>
@@ -7964,7 +8008,7 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H125" s="4" t="n">
         <v>0</v>
@@ -8023,7 +8067,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H126" s="2" t="n">
         <v>0</v>
@@ -8141,7 +8185,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H128" s="2" t="n">
         <v>6</v>
@@ -8204,7 +8248,7 @@
         </is>
       </c>
       <c r="G129" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H129" s="4" t="n">
         <v>1</v>
@@ -8267,7 +8311,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H130" s="2" t="n">
         <v>0</v>

</xml_diff>